<commit_message>
Admin: edit data/testimonials.xlsx via table editor
</commit_message>
<xml_diff>
--- a/data/testimonials.xlsx
+++ b/data/testimonials.xlsx
@@ -1,46 +1,55 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testimonials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Testimonials" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0056127D"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,82 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
@@ -209,6 +150,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -243,6 +185,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -277,20 +220,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -412,145 +351,137 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Show Profile Picture</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Profile Image URL</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Display Order</t>
-        </is>
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Active</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Show Profile Picture</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Testimonial</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Profile Image URL</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Display Order</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>संकल्प सदस्य</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>अविस्मरणीय दिवाळी… अविस्मरणीय टीम! 💫 संकल्प दिवाळी सोहळा यशस्वी होण्यामागे हाच खरा इन्क्रेडिबल ग्रुप — आपली संकल्प टीम! प्रत्येकाने आपला वेळ, श्रम आणि मनापासून दिलेला सहभाग या कार्यक्रमाचं खरं सौंदर्य बनलं. आपल्या एकोप्याने, सर्जनशीलतेने आणि न थकणाऱ्या उत्साहाने दिवाळीचा प्रकाश आणखी उजळला! मनःपूर्वक धन्यवाद या अद्भुत टीमला — तुमच्याशिवाय हा सोहळा इतका सुंदर झाला नसता! ✨</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A2" t="str">
+        <v xml:space="preserve">संकल्प सदस्य संकल्प सदस्य संकल्प सदस्य </v>
+      </c>
+      <c r="B2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C2" t="str">
+        <v>NO</v>
+      </c>
+      <c r="D2" t="str">
+        <v>अविस्मरणीय दिवाळी… अविस्मरणीय टीम!  संकल्प दिवाळी सोहळा यशस्वी होण्यामागे हाच खरा इन्क्रेडिबल ग्रुप — आपली संकल्प टीम! प्रत्येकाने आपला वेळ, श्रम आणि मनापासून दिलेला सहभाग या कार्यक्रमाचं खरं सौंदर्य बनलं. आपल्या एकोप्याने, सर्जनशीलतेने आणि न थकणाऱ्या उत्साहाने दिवाळीचा प्रकाश आणखी उजळला! मनःपूर्वक धन्यवाद या अद्भुत टीमला — तुमच्याशिवाय हा सोहळा इतका सुंदर झाला नसता! ✨</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Community Member</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>On this thanksgiving day, I would like to thank Sankalp Marathi Mandal for their tireless efforts in building a strong and supportive community!!! Hats off to you!! Apla Sanklap group has become a go-to platform for seeking help on any issue / problem / need / question — be it a passport and visa-related queries or job searches and even critical illnesses. It's amazing to see how Sankalp has created a sense of community and belonging. Its like a big family always being there for you. A big thank you to everyone in this community, and especially to the core members !!!</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A3" t="str">
+        <v>Community Member</v>
+      </c>
+      <c r="B3" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C3" t="str">
+        <v>NO</v>
+      </c>
+      <c r="D3" t="str">
+        <v>On this thanksgiving day, I would like to thank Sankalp Marathi Mandal for their tireless efforts in building a strong and supportive community!!! Hats off to you!! Apla Sanklap group has become a go-to platform for seeking help on any issue / problem / need / question — be it a passport and visa-related queries or job searches and even critical illnesses. It's amazing to see how Sankalp has created a sense of community and belonging. Its like a big family always being there for you. A big thank you to everyone in this community, and especially to the core members !!!</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>संकल्प सदस्य</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>यंदाचा संकल्प दिवाळी सोहळा अगदी वेगळा ठरला — हा फक्त कार्यक्रम नव्हता, तर एक आपुलकीचा अनुभव होता. स्थळाच्या मोकळ्या वातावरणामुळे सगळ्यांना एकमेकांशी संवाद साधता आला, हसता खेळता गप्पा मारता आल्या, आणि कार्यक्रम खरंच घरगुती पणातला सोहळा बनला. मी अनेक संकल्प आणि इतर संस्था आयोजित कार्यक्रम पाहिले आहेत, पण यंदाचा अनुभव खास होता — कारण प्रत्येकाला आपुलकीचा भाव जाणवला. हे खरंच फॅमिली कनेक्टेड इव्हेंट होतं! सर्वात कौतुकास्पद गोष्ट म्हणजे — अगदी थोड्या वेळात आपल्या मुलांनी, आजी-आजोबांनी, आणि संपूर्ण टीमने एकत्र येऊन तयारी केली आणि सुंदर सादरीकरणं केली. हीच खरी संकल्पची ताकद आहे — एकोप्याची आणि उत्साहाची! मनःपूर्वक धन्यवाद या सुंदर संध्याकाळीला संस्मरणीय बनवणाऱ्या प्रत्येकाला!</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="A4" t="str">
+        <v>संकल्प सदस्य</v>
+      </c>
+      <c r="B4" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C4" t="str">
+        <v>NO</v>
+      </c>
+      <c r="D4" t="str">
+        <v>यंदाचा संकल्प दिवाळी सोहळा अगदी वेगळा ठरला — हा फक्त कार्यक्रम नव्हता, तर एक आपुलकीचा अनुभव होता. स्थळाच्या मोकळ्या वातावरणामुळे सगळ्यांना एकमेकांशी संवाद साधता आला, हसता खेळता गप्पा मारता आल्या, आणि कार्यक्रम खरंच घरगुती पणातला सोहळा बनला. मी अनेक संकल्प आणि इतर संस्था आयोजित कार्यक्रम पाहिले आहेत, पण यंदाचा अनुभव खास होता — कारण प्रत्येकाला आपुलकीचा भाव जाणवला. हे खरंच फॅमिली कनेक्टेड इव्हेंट होतं! सर्वात कौतुकास्पद गोष्ट म्हणजे — अगदी थोड्या वेळात आपल्या मुलांनी, आजी-आजोबांनी, आणि संपूर्ण टीमने एकत्र येऊन तयारी केली आणि सुंदर सादरीकरणं केली. हीच खरी संकल्पची ताकद आहे — एकोप्याची आणि उत्साहाची! मनःपूर्वक धन्यवाद या सुंदर संध्याकाळीला संस्मरणीय बनवणाऱ्या प्रत्येकाला!</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>